<commit_message>
Added new RDF data schemes and visual schemes for environment-table11-12, and fixed XLSX spreadsheet for environment-table12
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table12.xlsx
+++ b/sources/table_normalization/xlsx/environment-table12.xlsx
@@ -1039,42 +1039,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="12" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1108,16 +1072,9 @@
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="16" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1128,11 +1085,29 @@
     <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="165" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="15" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1143,12 +1118,37 @@
     <xf numFmtId="165" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -1456,7 +1456,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4226,13 +4226,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:49" ht="14.5">
-      <c r="A1" s="81" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:49">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="70" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
@@ -4242,230 +4242,230 @@
       <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:49" s="5" customFormat="1" ht="18">
-      <c r="A4" s="92" t="s">
+      <c r="A4" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="99" t="s">
+      <c r="B4" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="100"/>
-      <c r="D4" s="100"/>
-      <c r="E4" s="100"/>
-      <c r="F4" s="101"/>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
-      <c r="I4" s="101"/>
-      <c r="J4" s="101"/>
-      <c r="K4" s="101"/>
-      <c r="L4" s="102"/>
-      <c r="M4" s="99"/>
-      <c r="N4" s="99"/>
-      <c r="O4" s="99"/>
-      <c r="P4" s="101"/>
-      <c r="Q4" s="101"/>
-      <c r="R4" s="101"/>
-      <c r="S4" s="101"/>
-      <c r="T4" s="101"/>
-      <c r="U4" s="101"/>
-      <c r="V4" s="101"/>
-      <c r="W4" s="101"/>
-      <c r="X4" s="101"/>
-      <c r="Y4" s="101"/>
-      <c r="Z4" s="101"/>
-      <c r="AA4" s="101"/>
-      <c r="AB4" s="101"/>
-      <c r="AC4" s="101"/>
-      <c r="AD4" s="101"/>
-      <c r="AE4" s="101"/>
-      <c r="AF4" s="103" t="s">
+      <c r="C4" s="83"/>
+      <c r="D4" s="83"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
+      <c r="I4" s="84"/>
+      <c r="J4" s="84"/>
+      <c r="K4" s="84"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="82"/>
+      <c r="O4" s="82"/>
+      <c r="P4" s="84"/>
+      <c r="Q4" s="84"/>
+      <c r="R4" s="84"/>
+      <c r="S4" s="84"/>
+      <c r="T4" s="84"/>
+      <c r="U4" s="84"/>
+      <c r="V4" s="84"/>
+      <c r="W4" s="84"/>
+      <c r="X4" s="84"/>
+      <c r="Y4" s="84"/>
+      <c r="Z4" s="84"/>
+      <c r="AA4" s="84"/>
+      <c r="AB4" s="84"/>
+      <c r="AC4" s="84"/>
+      <c r="AD4" s="84"/>
+      <c r="AE4" s="84"/>
+      <c r="AF4" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="AG4" s="102"/>
-      <c r="AH4" s="104"/>
-      <c r="AI4" s="102"/>
-      <c r="AJ4" s="102"/>
-      <c r="AK4" s="102"/>
-      <c r="AL4" s="101"/>
-      <c r="AM4" s="101"/>
-      <c r="AN4" s="101"/>
-      <c r="AO4" s="101"/>
-      <c r="AP4" s="101"/>
-      <c r="AQ4" s="101"/>
-      <c r="AR4" s="101"/>
-      <c r="AS4" s="101"/>
-      <c r="AT4" s="101"/>
-      <c r="AU4" s="107" t="s">
+      <c r="AG4" s="85"/>
+      <c r="AH4" s="87"/>
+      <c r="AI4" s="85"/>
+      <c r="AJ4" s="85"/>
+      <c r="AK4" s="85"/>
+      <c r="AL4" s="84"/>
+      <c r="AM4" s="84"/>
+      <c r="AN4" s="84"/>
+      <c r="AO4" s="84"/>
+      <c r="AP4" s="84"/>
+      <c r="AQ4" s="84"/>
+      <c r="AR4" s="84"/>
+      <c r="AS4" s="84"/>
+      <c r="AT4" s="84"/>
+      <c r="AU4" s="96" t="s">
         <v>5</v>
       </c>
-      <c r="AV4" s="108"/>
-      <c r="AW4" s="109"/>
+      <c r="AV4" s="97"/>
+      <c r="AW4" s="98"/>
     </row>
     <row r="5" spans="1:49" s="9" customFormat="1" ht="29.25" customHeight="1">
-      <c r="A5" s="93"/>
-      <c r="B5" s="75" t="s">
+      <c r="A5" s="110"/>
+      <c r="B5" s="99" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="75"/>
-      <c r="D5" s="76"/>
-      <c r="E5" s="77" t="s">
+      <c r="C5" s="99"/>
+      <c r="D5" s="100"/>
+      <c r="E5" s="101" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="75"/>
-      <c r="G5" s="76"/>
-      <c r="H5" s="77" t="s">
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
+      <c r="H5" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="75"/>
-      <c r="J5" s="76"/>
-      <c r="K5" s="77" t="s">
+      <c r="I5" s="99"/>
+      <c r="J5" s="100"/>
+      <c r="K5" s="101" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="75"/>
-      <c r="M5" s="76"/>
-      <c r="N5" s="77" t="s">
+      <c r="L5" s="99"/>
+      <c r="M5" s="100"/>
+      <c r="N5" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="O5" s="75"/>
-      <c r="P5" s="76"/>
+      <c r="O5" s="99"/>
+      <c r="P5" s="100"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="7" t="s">
         <v>11</v>
       </c>
       <c r="S5" s="8"/>
-      <c r="T5" s="77" t="s">
+      <c r="T5" s="101" t="s">
         <v>12</v>
       </c>
-      <c r="U5" s="75"/>
-      <c r="V5" s="76"/>
-      <c r="W5" s="77" t="s">
+      <c r="U5" s="99"/>
+      <c r="V5" s="100"/>
+      <c r="W5" s="101" t="s">
         <v>13</v>
       </c>
-      <c r="X5" s="75"/>
-      <c r="Y5" s="76"/>
-      <c r="Z5" s="78" t="s">
+      <c r="X5" s="99"/>
+      <c r="Y5" s="100"/>
+      <c r="Z5" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="AA5" s="79"/>
-      <c r="AB5" s="80"/>
-      <c r="AC5" s="78" t="s">
+      <c r="AA5" s="103"/>
+      <c r="AB5" s="104"/>
+      <c r="AC5" s="102" t="s">
         <v>15</v>
       </c>
-      <c r="AD5" s="75"/>
-      <c r="AE5" s="76"/>
-      <c r="AF5" s="69" t="s">
+      <c r="AD5" s="99"/>
+      <c r="AE5" s="100"/>
+      <c r="AF5" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="AG5" s="70"/>
-      <c r="AH5" s="71"/>
-      <c r="AI5" s="69" t="s">
+      <c r="AG5" s="91"/>
+      <c r="AH5" s="92"/>
+      <c r="AI5" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="AJ5" s="70"/>
-      <c r="AK5" s="71"/>
-      <c r="AL5" s="69" t="s">
+      <c r="AJ5" s="91"/>
+      <c r="AK5" s="92"/>
+      <c r="AL5" s="90" t="s">
         <v>18</v>
       </c>
-      <c r="AM5" s="70"/>
-      <c r="AN5" s="71"/>
-      <c r="AO5" s="69" t="s">
+      <c r="AM5" s="91"/>
+      <c r="AN5" s="92"/>
+      <c r="AO5" s="90" t="s">
         <v>19</v>
       </c>
-      <c r="AP5" s="70"/>
-      <c r="AQ5" s="71"/>
-      <c r="AR5" s="69" t="s">
+      <c r="AP5" s="91"/>
+      <c r="AQ5" s="92"/>
+      <c r="AR5" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="AS5" s="70"/>
-      <c r="AT5" s="71"/>
-      <c r="AU5" s="72"/>
-      <c r="AV5" s="73"/>
-      <c r="AW5" s="74"/>
+      <c r="AS5" s="91"/>
+      <c r="AT5" s="92"/>
+      <c r="AU5" s="93"/>
+      <c r="AV5" s="94"/>
+      <c r="AW5" s="95"/>
     </row>
     <row r="6" spans="1:49" s="10" customFormat="1">
-      <c r="A6" s="94"/>
-      <c r="B6" s="96" t="s">
+      <c r="A6" s="111"/>
+      <c r="B6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="96" t="s">
+      <c r="C6" s="108"/>
+      <c r="D6" s="109"/>
+      <c r="E6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="105"/>
-      <c r="G6" s="106"/>
-      <c r="H6" s="96" t="s">
+      <c r="F6" s="106"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="105"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="96" t="s">
+      <c r="I6" s="106"/>
+      <c r="J6" s="107"/>
+      <c r="K6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="105"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="96" t="s">
+      <c r="L6" s="106"/>
+      <c r="M6" s="107"/>
+      <c r="N6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="O6" s="105"/>
-      <c r="P6" s="106"/>
-      <c r="Q6" s="96" t="s">
+      <c r="O6" s="106"/>
+      <c r="P6" s="107"/>
+      <c r="Q6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="105"/>
-      <c r="S6" s="106"/>
-      <c r="T6" s="96" t="s">
+      <c r="R6" s="106"/>
+      <c r="S6" s="107"/>
+      <c r="T6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="U6" s="105"/>
-      <c r="V6" s="106"/>
-      <c r="W6" s="96" t="s">
+      <c r="U6" s="106"/>
+      <c r="V6" s="107"/>
+      <c r="W6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="X6" s="105"/>
-      <c r="Y6" s="106"/>
-      <c r="Z6" s="96" t="s">
+      <c r="X6" s="106"/>
+      <c r="Y6" s="107"/>
+      <c r="Z6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AA6" s="105"/>
-      <c r="AB6" s="106"/>
-      <c r="AC6" s="96" t="s">
+      <c r="AA6" s="106"/>
+      <c r="AB6" s="107"/>
+      <c r="AC6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AD6" s="105"/>
-      <c r="AE6" s="106"/>
-      <c r="AF6" s="96" t="s">
+      <c r="AD6" s="106"/>
+      <c r="AE6" s="107"/>
+      <c r="AF6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AG6" s="105"/>
-      <c r="AH6" s="106"/>
-      <c r="AI6" s="96" t="s">
+      <c r="AG6" s="106"/>
+      <c r="AH6" s="107"/>
+      <c r="AI6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AJ6" s="105"/>
-      <c r="AK6" s="106"/>
-      <c r="AL6" s="96" t="s">
+      <c r="AJ6" s="106"/>
+      <c r="AK6" s="107"/>
+      <c r="AL6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AM6" s="105"/>
-      <c r="AN6" s="106"/>
-      <c r="AO6" s="96" t="s">
+      <c r="AM6" s="106"/>
+      <c r="AN6" s="107"/>
+      <c r="AO6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AP6" s="105"/>
-      <c r="AQ6" s="106"/>
-      <c r="AR6" s="96" t="s">
+      <c r="AP6" s="106"/>
+      <c r="AQ6" s="107"/>
+      <c r="AR6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AS6" s="105"/>
-      <c r="AT6" s="106"/>
-      <c r="AU6" s="96" t="s">
+      <c r="AS6" s="106"/>
+      <c r="AT6" s="107"/>
+      <c r="AU6" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="AV6" s="105"/>
-      <c r="AW6" s="106"/>
+      <c r="AV6" s="106"/>
+      <c r="AW6" s="107"/>
     </row>
     <row r="7" spans="1:49" s="18" customFormat="1">
-      <c r="A7" s="95" t="s">
+      <c r="A7" s="81" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="11">
@@ -4474,7 +4474,7 @@
       <c r="C7" s="12">
         <v>2008</v>
       </c>
-      <c r="D7" s="110" t="s">
+      <c r="D7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="E7" s="11">
@@ -4483,7 +4483,7 @@
       <c r="F7" s="12">
         <v>2008</v>
       </c>
-      <c r="G7" s="110" t="s">
+      <c r="G7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="H7" s="11">
@@ -4492,7 +4492,7 @@
       <c r="I7" s="12">
         <v>2008</v>
       </c>
-      <c r="J7" s="110" t="s">
+      <c r="J7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="K7" s="11">
@@ -4501,7 +4501,7 @@
       <c r="L7" s="12">
         <v>2008</v>
       </c>
-      <c r="M7" s="110" t="s">
+      <c r="M7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="N7" s="11">
@@ -4510,7 +4510,7 @@
       <c r="O7" s="12">
         <v>2008</v>
       </c>
-      <c r="P7" s="110" t="s">
+      <c r="P7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="Q7" s="11">
@@ -4519,7 +4519,7 @@
       <c r="R7" s="12">
         <v>2008</v>
       </c>
-      <c r="S7" s="110" t="s">
+      <c r="S7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="T7" s="11">
@@ -4528,7 +4528,7 @@
       <c r="U7" s="12">
         <v>2008</v>
       </c>
-      <c r="V7" s="110" t="s">
+      <c r="V7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="W7" s="11">
@@ -4537,7 +4537,7 @@
       <c r="X7" s="12">
         <v>2008</v>
       </c>
-      <c r="Y7" s="110" t="s">
+      <c r="Y7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="Z7" s="11">
@@ -4546,7 +4546,7 @@
       <c r="AA7" s="12">
         <v>2008</v>
       </c>
-      <c r="AB7" s="110" t="s">
+      <c r="AB7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="AC7" s="11">
@@ -4555,7 +4555,7 @@
       <c r="AD7" s="12">
         <v>2008</v>
       </c>
-      <c r="AE7" s="111" t="s">
+      <c r="AE7" s="89" t="s">
         <v>23</v>
       </c>
       <c r="AF7" s="13">
@@ -4564,7 +4564,7 @@
       <c r="AG7" s="14">
         <v>2008</v>
       </c>
-      <c r="AH7" s="110" t="s">
+      <c r="AH7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="AI7" s="13">
@@ -4573,7 +4573,7 @@
       <c r="AJ7" s="14">
         <v>2008</v>
       </c>
-      <c r="AK7" s="110" t="s">
+      <c r="AK7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="AL7" s="13">
@@ -4582,7 +4582,7 @@
       <c r="AM7" s="14">
         <v>2008</v>
       </c>
-      <c r="AN7" s="110" t="s">
+      <c r="AN7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="AO7" s="13">
@@ -4591,7 +4591,7 @@
       <c r="AP7" s="14">
         <v>2008</v>
       </c>
-      <c r="AQ7" s="110" t="s">
+      <c r="AQ7" s="88" t="s">
         <v>23</v>
       </c>
       <c r="AR7" s="13">
@@ -4609,7 +4609,7 @@
       <c r="AV7" s="17">
         <v>2008</v>
       </c>
-      <c r="AW7" s="110" t="s">
+      <c r="AW7" s="88" t="s">
         <v>23</v>
       </c>
     </row>
@@ -20220,7 +20220,7 @@
       </c>
     </row>
     <row r="118" spans="1:49" s="42" customFormat="1">
-      <c r="A118" s="83" t="s">
+      <c r="A118" s="71" t="s">
         <v>129</v>
       </c>
       <c r="B118" s="57"/>
@@ -20273,7 +20273,7 @@
       <c r="AW118"/>
     </row>
     <row r="119" spans="1:49" s="42" customFormat="1">
-      <c r="A119" s="84" t="s">
+      <c r="A119" s="72" t="s">
         <v>130</v>
       </c>
       <c r="B119" s="59"/>
@@ -20326,7 +20326,7 @@
       <c r="AW119"/>
     </row>
     <row r="120" spans="1:49" s="42" customFormat="1">
-      <c r="A120" s="85" t="s">
+      <c r="A120" s="73" t="s">
         <v>131</v>
       </c>
       <c r="B120" s="60"/>
@@ -20379,7 +20379,7 @@
       <c r="AW120"/>
     </row>
     <row r="121" spans="1:49" s="42" customFormat="1">
-      <c r="A121" s="86" t="s">
+      <c r="A121" s="74" t="s">
         <v>132</v>
       </c>
       <c r="B121" s="62"/>
@@ -20432,7 +20432,7 @@
       <c r="AW121" s="63"/>
     </row>
     <row r="122" spans="1:49" s="42" customFormat="1">
-      <c r="A122" s="86" t="s">
+      <c r="A122" s="74" t="s">
         <v>133</v>
       </c>
       <c r="B122" s="62"/>
@@ -20485,7 +20485,7 @@
       <c r="AW122" s="63"/>
     </row>
     <row r="123" spans="1:49" s="42" customFormat="1">
-      <c r="A123" s="87" t="s">
+      <c r="A123" s="75" t="s">
         <v>134</v>
       </c>
       <c r="B123" s="62"/>
@@ -20589,7 +20589,7 @@
       <c r="AW124" s="63"/>
     </row>
     <row r="125" spans="1:49" s="42" customFormat="1">
-      <c r="A125" s="83" t="s">
+      <c r="A125" s="71" t="s">
         <v>135</v>
       </c>
       <c r="B125" s="57"/>
@@ -20642,7 +20642,7 @@
       <c r="AW125"/>
     </row>
     <row r="126" spans="1:49" s="42" customFormat="1">
-      <c r="A126" s="83" t="s">
+      <c r="A126" s="71" t="s">
         <v>136</v>
       </c>
       <c r="B126" s="57"/>
@@ -20695,7 +20695,7 @@
       <c r="AW126"/>
     </row>
     <row r="127" spans="1:49" s="42" customFormat="1">
-      <c r="A127" s="83" t="s">
+      <c r="A127" s="71" t="s">
         <v>137</v>
       </c>
       <c r="B127" s="57"/>
@@ -20799,7 +20799,7 @@
       <c r="AW128"/>
     </row>
     <row r="129" spans="1:15">
-      <c r="A129" s="88" t="s">
+      <c r="A129" s="76" t="s">
         <v>138</v>
       </c>
       <c r="B129" s="65"/>
@@ -20812,7 +20812,7 @@
       <c r="O129" s="66"/>
     </row>
     <row r="130" spans="1:15">
-      <c r="A130" s="89" t="s">
+      <c r="A130" s="77" t="s">
         <v>139</v>
       </c>
       <c r="B130" s="65"/>
@@ -20823,7 +20823,7 @@
       <c r="G130"/>
     </row>
     <row r="131" spans="1:15">
-      <c r="A131" s="89" t="s">
+      <c r="A131" s="77" t="s">
         <v>140</v>
       </c>
       <c r="B131" s="65"/>
@@ -20834,7 +20834,7 @@
       <c r="G131"/>
     </row>
     <row r="132" spans="1:15">
-      <c r="A132" s="89" t="s">
+      <c r="A132" s="77" t="s">
         <v>141</v>
       </c>
       <c r="B132" s="65"/>
@@ -20845,7 +20845,7 @@
       <c r="G132"/>
     </row>
     <row r="133" spans="1:15">
-      <c r="A133" s="89" t="s">
+      <c r="A133" s="77" t="s">
         <v>142</v>
       </c>
       <c r="B133" s="65"/>
@@ -20856,7 +20856,7 @@
       <c r="G133"/>
     </row>
     <row r="134" spans="1:15">
-      <c r="A134" s="90" t="s">
+      <c r="A134" s="78" t="s">
         <v>143</v>
       </c>
       <c r="B134" s="65"/>
@@ -20876,13 +20876,33 @@
       <c r="G135"/>
     </row>
     <row r="136" spans="1:15">
-      <c r="A136" s="91" t="s">
+      <c r="A136" s="79" t="s">
         <v>144</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A7:A117"/>
   <mergeCells count="32">
+    <mergeCell ref="AR6:AT6"/>
+    <mergeCell ref="AU6:AW6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
+    <mergeCell ref="Z6:AB6"/>
+    <mergeCell ref="AC6:AE6"/>
+    <mergeCell ref="AF6:AH6"/>
+    <mergeCell ref="AI6:AK6"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="Q6:S6"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AL6:AN6"/>
+    <mergeCell ref="AO6:AQ6"/>
     <mergeCell ref="AR5:AT5"/>
     <mergeCell ref="AU5:AW5"/>
     <mergeCell ref="AU4:AW4"/>
@@ -20895,26 +20915,6 @@
     <mergeCell ref="W5:Y5"/>
     <mergeCell ref="Z5:AB5"/>
     <mergeCell ref="AC5:AE5"/>
-    <mergeCell ref="Q6:S6"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="K6:M6"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="AL6:AN6"/>
-    <mergeCell ref="AO6:AQ6"/>
-    <mergeCell ref="AR6:AT6"/>
-    <mergeCell ref="AU6:AW6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="Z6:AB6"/>
-    <mergeCell ref="AC6:AE6"/>
-    <mergeCell ref="AF6:AH6"/>
-    <mergeCell ref="AI6:AK6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>

</xml_diff>